<commit_message>
more keyword matches, simplify insurance
</commit_message>
<xml_diff>
--- a/Budget.xlsx
+++ b/Budget.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/572d0a92ad25842f/Documents/Budget API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{79BB131A-79AE-42EF-86EF-ED73B9B6A30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{763E49E8-2A5C-4749-84ED-31D8139FE7A0}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{79BB131A-79AE-42EF-86EF-ED73B9B6A30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B94CF90-6365-4DCD-AFA3-730CA2BF03C3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>Net Income Per Month</t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>Eating out</t>
+  </si>
+  <si>
+    <t>Therapy</t>
   </si>
 </sst>
 </file>
@@ -879,8 +882,8 @@
         <v>5</v>
       </c>
       <c r="B2" s="3">
-        <f>23*40*0.817*4</f>
-        <v>3006.56</v>
+        <f>23*40*0.75*4</f>
+        <v>2760</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>6</v>
@@ -968,7 +971,7 @@
       </c>
       <c r="E5" s="3">
         <f>SUM(H2:H16)</f>
-        <v>890.96416666666676</v>
+        <v>927.12333333333333</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>18</v>
@@ -983,7 +986,7 @@
       </c>
       <c r="B6" s="24">
         <f>SUM(B2:B5)</f>
-        <v>6678.5599999999995</v>
+        <v>6432</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>20</v>
@@ -1025,7 +1028,7 @@
       </c>
       <c r="H8" s="3">
         <f>K14</f>
-        <v>333.84083333333331</v>
+        <v>350</v>
       </c>
       <c r="J8" s="20" t="s">
         <v>50</v>
@@ -1076,7 +1079,7 @@
       </c>
       <c r="E10" s="3">
         <f>SUM(H19:H20)</f>
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>29</v>
@@ -1100,14 +1103,14 @@
       </c>
       <c r="B11" s="23">
         <f>B6</f>
-        <v>6678.5599999999995</v>
+        <v>6432</v>
       </c>
       <c r="D11" s="26" t="s">
         <v>27</v>
       </c>
       <c r="E11" s="27">
         <f>SUM(E2:E10)</f>
-        <v>5715.9641666666666</v>
+        <v>5452.123333333333</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>31</v>
@@ -1132,7 +1135,7 @@
       </c>
       <c r="B12" s="25">
         <f>E11</f>
-        <v>5715.9641666666666</v>
+        <v>5452.123333333333</v>
       </c>
       <c r="D12" s="10"/>
       <c r="G12" s="3" t="s">
@@ -1158,7 +1161,7 @@
       </c>
       <c r="B13" s="28">
         <f>B11-B12</f>
-        <v>962.59583333333285</v>
+        <v>979.87666666666701</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>35</v>
@@ -1199,8 +1202,7 @@
         <v>27</v>
       </c>
       <c r="K14" s="19">
-        <f>SUM(K9:K13)</f>
-        <v>333.84083333333331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="14">
@@ -1239,8 +1241,12 @@
         <f>H11</f>
         <v>10.833333333333334</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="6"/>
+      <c r="G16" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" s="6">
+        <v>20</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="15.75" customHeight="1">
       <c r="A17" s="11">
@@ -1308,7 +1314,7 @@
         <v>45</v>
       </c>
       <c r="H20" s="6">
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15.75" customHeight="1">
@@ -1586,7 +1592,7 @@
       </c>
       <c r="H2" s="36">
         <f>Sheet1!B11</f>
-        <v>6678.5599999999995</v>
+        <v>6432</v>
       </c>
       <c r="J2" s="34" t="str">
         <f>Sheet1!G2</f>
@@ -1644,7 +1650,7 @@
       </c>
       <c r="H3" s="29">
         <f>Sheet1!B12</f>
-        <v>5715.9641666666666</v>
+        <v>5452.123333333333</v>
       </c>
       <c r="J3" s="34" t="str">
         <f>Sheet1!G3</f>
@@ -1676,7 +1682,7 @@
       </c>
       <c r="T3" s="30">
         <f>Sheet1!H20</f>
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="13" thickBot="1">
@@ -1702,7 +1708,7 @@
       </c>
       <c r="H4" s="30">
         <f>Sheet1!B13</f>
-        <v>962.59583333333285</v>
+        <v>979.87666666666701</v>
       </c>
       <c r="J4" s="34" t="str">
         <f>Sheet1!G4</f>
@@ -1736,7 +1742,7 @@
       </c>
       <c r="B5" s="29">
         <f>Sheet1!E5</f>
-        <v>890.96416666666676</v>
+        <v>927.12333333333333</v>
       </c>
       <c r="D5" s="33" t="str">
         <f>Sheet1!D17</f>
@@ -1810,13 +1816,12 @@
         <f>Sheet1!H7</f>
         <v>10</v>
       </c>
-      <c r="M7" s="33" t="str">
-        <f>Sheet1!J14</f>
-        <v>Total</v>
+      <c r="M7" s="33" t="s">
+        <v>50</v>
       </c>
       <c r="N7" s="31">
         <f>Sheet1!K14</f>
-        <v>333.84083333333331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" spans="1:20">
@@ -1834,7 +1839,7 @@
       </c>
       <c r="K8" s="29">
         <f>Sheet1!H8</f>
-        <v>333.84083333333331</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9" spans="1:20">
@@ -1862,7 +1867,7 @@
       </c>
       <c r="B10" s="29">
         <f>Sheet1!E10</f>
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="J10" s="34" t="str">
         <f>Sheet1!G10</f>
@@ -1880,7 +1885,7 @@
       </c>
       <c r="B11" s="31">
         <f>Sheet1!E11</f>
-        <v>5715.9641666666666</v>
+        <v>5452.123333333333</v>
       </c>
       <c r="J11" s="34" t="str">
         <f>Sheet1!G11</f>
@@ -1932,13 +1937,13 @@
       </c>
     </row>
     <row r="16" spans="1:20" ht="13" thickBot="1">
-      <c r="J16" s="34">
+      <c r="J16" s="34" t="str">
         <f>Sheet1!G16</f>
-        <v>0</v>
+        <v>Therapy</v>
       </c>
       <c r="K16" s="29">
         <f>Sheet1!H16</f>
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="10:11" ht="13" thickBot="1">
@@ -1947,7 +1952,7 @@
       </c>
       <c r="K17" s="31">
         <f>SUM(K2:K16)</f>
-        <v>890.96416666666676</v>
+        <v>927.12333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>